<commit_message>
shortcuts for main actions
</commit_message>
<xml_diff>
--- a/JavaApplication1/pruebach.xlsx
+++ b/JavaApplication1/pruebach.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="50">
   <si>
     <t>markIn</t>
   </si>
@@ -44,37 +44,88 @@
     <t>fps</t>
   </si>
   <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>13:02:28:452</t>
+  </si>
+  <si>
+    <t>na</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>dsfsdfsdfdsf</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>29.97d</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t>13:00:11:814</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>008</t>
+  </si>
+  <si>
+    <t>13:00:11:295</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>12:57:00:387</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>12:56:40:58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGJHGJHG </t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
     <t>005</t>
   </si>
   <si>
     <t>21:40:22:742</t>
   </si>
   <si>
-    <t>na</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>SDFSDFS</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
-    <t>FALSE</t>
-  </si>
-  <si>
-    <t>29.97d</t>
-  </si>
-  <si>
     <t>004</t>
   </si>
   <si>
     <t>21:35:47:727</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>4</t>
@@ -170,7 +221,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -324,16 +375,16 @@
         <v>13</v>
       </c>
       <c r="E5" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H5" t="s" s="2">
         <v>27</v>
-      </c>
-      <c r="F5" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s" s="2">
-        <v>28</v>
       </c>
       <c r="I5" t="n" s="2">
         <v>0.0</v>
@@ -347,36 +398,211 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="B6" t="s" s="2">
+      <c r="C6" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="C6" t="s" s="2">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E6" t="s" s="2">
+      <c r="F6" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="F6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s" s="2">
+      <c r="I6" t="n" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="J6" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="K6" t="s" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="I6" t="n" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="J6" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="K6" t="s" s="2">
+      <c r="B7" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H7" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="I7" t="n" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="J7" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="K7" t="s" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="I8" t="n" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="J8" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="K8" t="s" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="2">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="F9" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H9" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="I9" t="n" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="J9" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="K9" t="s" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s" s="2">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s" s="2">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G10" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H10" t="s" s="2">
+        <v>45</v>
+      </c>
+      <c r="I10" t="n" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="J10" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="K10" t="s" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="2">
+        <v>46</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>47</v>
+      </c>
+      <c r="C11" t="s" s="2">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="F11" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="H11" t="s" s="2">
+        <v>49</v>
+      </c>
+      <c r="I11" t="n" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="J11" t="s" s="2">
+        <v>16</v>
+      </c>
+      <c r="K11" t="s" s="2">
         <v>17</v>
       </c>
     </row>

</xml_diff>